<commit_message>
B46 finding 4 logged: import splits cash lines into per-type accounts; txn-picker local naming makes identical chips — walk row 22 proposed (shared naming) + founder double-count check
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build46-feedback-v1-2026-07-29.xlsx
+++ b/docs/FCC-core-55-70/build46-feedback-v1-2026-07-29.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -571,6 +571,31 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="130" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Record-a-transaction: the account picker shows "E*Trade savings" three times + "E*Trade brokerage" once — you only uploaded one account</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED: your statement upload deliberately splits by type — LCTX became a brokerage account, and every CASH-type line on the file (money market / sweep / CD-like rows) became its OWN small account, each filed under Cash with institution E*Trade. Three cash lines → three accounts. The picker then names chips its own local way (institution first; on a name collision it appends the TYPE) instead of the shared account-naming helper the rest of the app uses — three accounts sharing institution AND type = three IDENTICAL chips. A one-concept-one-helper violation (same class as your B43 finding 9).</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Fix (a): the picker adopts the shared account naming — you would see the real names (e.g. the fund name, "· 1 / · 2") instead of three clones. Proposed as Build-47 walk row 22 (conforms to the approved naming system, no new design). Check (b) FOR YOU: those three accounts may DOUBLE-COUNT money your live E*TRADE connection already reports — open Net worth → the Cash class (or the new By-institution pill) and look at their names and amounts; if they duplicate connected money, they should be deleted. Tell me what you see and I will guide or script the cleanup.</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>FIX PROPOSED + your 30-sec check</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>